<commit_message>
data: sync PC-server-0148 2026-10-21 08:04
</commit_message>
<xml_diff>
--- a/data/飞猪.xlsx
+++ b/data/飞猪.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R408"/>
+  <dimension ref="A1:R413"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30415,15 +30415,11 @@
           <t>向上航服</t>
         </is>
       </c>
-      <c r="C400" t="inlineStr">
-        <is>
-          <t>5184</t>
-        </is>
-      </c>
-      <c r="D400" t="inlineStr">
-        <is>
-          <t>100745</t>
-        </is>
+      <c r="C400" t="n">
+        <v>5184</v>
+      </c>
+      <c r="D400" t="n">
+        <v>100745</v>
       </c>
       <c r="E400" t="inlineStr">
         <is>
@@ -30445,35 +30441,23 @@
           <t>系统异常,业务异常,未知异常</t>
         </is>
       </c>
-      <c r="I400" t="inlineStr">
-        <is>
-          <t>120</t>
-        </is>
-      </c>
-      <c r="J400" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="K400" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="L400" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="M400" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="N400" t="inlineStr">
-        <is>
-          <t>45</t>
-        </is>
+      <c r="I400" t="n">
+        <v>120</v>
+      </c>
+      <c r="J400" t="n">
+        <v>25</v>
+      </c>
+      <c r="K400" t="n">
+        <v>5</v>
+      </c>
+      <c r="L400" t="n">
+        <v>20</v>
+      </c>
+      <c r="M400" t="n">
+        <v>15</v>
+      </c>
+      <c r="N400" t="n">
+        <v>45</v>
       </c>
       <c r="O400" t="inlineStr">
         <is>
@@ -30507,15 +30491,11 @@
           <t>平安航旅</t>
         </is>
       </c>
-      <c r="C401" t="inlineStr">
-        <is>
-          <t>4470</t>
-        </is>
-      </c>
-      <c r="D401" t="inlineStr">
-        <is>
-          <t>138001</t>
-        </is>
+      <c r="C401" t="n">
+        <v>4470</v>
+      </c>
+      <c r="D401" t="n">
+        <v>138001</v>
       </c>
       <c r="E401" t="inlineStr">
         <is>
@@ -30537,35 +30517,23 @@
           <t>系统异常,业务异常,未知异常</t>
         </is>
       </c>
-      <c r="I401" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="J401" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="K401" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="L401" t="inlineStr">
-        <is>
-          <t>63</t>
-        </is>
-      </c>
-      <c r="M401" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="N401" t="inlineStr">
-        <is>
-          <t>45</t>
-        </is>
+      <c r="I401" t="n">
+        <v>60</v>
+      </c>
+      <c r="J401" t="n">
+        <v>11</v>
+      </c>
+      <c r="K401" t="n">
+        <v>7</v>
+      </c>
+      <c r="L401" t="n">
+        <v>63</v>
+      </c>
+      <c r="M401" t="n">
+        <v>60</v>
+      </c>
+      <c r="N401" t="n">
+        <v>45</v>
       </c>
       <c r="O401" t="inlineStr">
         <is>
@@ -30599,15 +30567,11 @@
           <t>向上航服</t>
         </is>
       </c>
-      <c r="C402" t="inlineStr">
-        <is>
-          <t>5184</t>
-        </is>
-      </c>
-      <c r="D402" t="inlineStr">
-        <is>
-          <t>100745</t>
-        </is>
+      <c r="C402" t="n">
+        <v>5184</v>
+      </c>
+      <c r="D402" t="n">
+        <v>100745</v>
       </c>
       <c r="E402" t="inlineStr">
         <is>
@@ -30629,35 +30593,23 @@
           <t>系统异常,业务异常,未知异常</t>
         </is>
       </c>
-      <c r="I402" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="J402" t="inlineStr">
-        <is>
-          <t>186</t>
-        </is>
-      </c>
-      <c r="K402" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="L402" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="M402" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="N402" t="inlineStr">
-        <is>
-          <t>45</t>
-        </is>
+      <c r="I402" t="n">
+        <v>60</v>
+      </c>
+      <c r="J402" t="n">
+        <v>186</v>
+      </c>
+      <c r="K402" t="n">
+        <v>30</v>
+      </c>
+      <c r="L402" t="n">
+        <v>16</v>
+      </c>
+      <c r="M402" t="n">
+        <v>15</v>
+      </c>
+      <c r="N402" t="n">
+        <v>45</v>
       </c>
       <c r="O402" t="inlineStr">
         <is>
@@ -30691,15 +30643,11 @@
           <t>向上航服</t>
         </is>
       </c>
-      <c r="C403" t="inlineStr">
-        <is>
-          <t>5184</t>
-        </is>
-      </c>
-      <c r="D403" t="inlineStr">
-        <is>
-          <t>100745</t>
-        </is>
+      <c r="C403" t="n">
+        <v>5184</v>
+      </c>
+      <c r="D403" t="n">
+        <v>100745</v>
       </c>
       <c r="E403" t="inlineStr">
         <is>
@@ -30721,35 +30669,23 @@
           <t>系统异常,业务异常,未知异常</t>
         </is>
       </c>
-      <c r="I403" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="J403" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="K403" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="L403" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="M403" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="N403" t="inlineStr">
-        <is>
-          <t>90</t>
-        </is>
+      <c r="I403" t="n">
+        <v>60</v>
+      </c>
+      <c r="J403" t="n">
+        <v>23</v>
+      </c>
+      <c r="K403" t="n">
+        <v>6</v>
+      </c>
+      <c r="L403" t="n">
+        <v>26</v>
+      </c>
+      <c r="M403" t="n">
+        <v>15</v>
+      </c>
+      <c r="N403" t="n">
+        <v>90</v>
       </c>
       <c r="O403" t="inlineStr">
         <is>
@@ -30783,15 +30719,11 @@
           <t>平安航旅</t>
         </is>
       </c>
-      <c r="C404" t="inlineStr">
-        <is>
-          <t>4470</t>
-        </is>
-      </c>
-      <c r="D404" t="inlineStr">
-        <is>
-          <t>138001</t>
-        </is>
+      <c r="C404" t="n">
+        <v>4470</v>
+      </c>
+      <c r="D404" t="n">
+        <v>138001</v>
       </c>
       <c r="E404" t="inlineStr">
         <is>
@@ -30813,35 +30745,23 @@
           <t>系统异常,业务异常,未知异常</t>
         </is>
       </c>
-      <c r="I404" t="inlineStr">
-        <is>
-          <t>120</t>
-        </is>
-      </c>
-      <c r="J404" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
-      </c>
-      <c r="K404" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="L404" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="M404" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="N404" t="inlineStr">
-        <is>
-          <t>45</t>
-        </is>
+      <c r="I404" t="n">
+        <v>120</v>
+      </c>
+      <c r="J404" t="n">
+        <v>31</v>
+      </c>
+      <c r="K404" t="n">
+        <v>8</v>
+      </c>
+      <c r="L404" t="n">
+        <v>25</v>
+      </c>
+      <c r="M404" t="n">
+        <v>20</v>
+      </c>
+      <c r="N404" t="n">
+        <v>45</v>
       </c>
       <c r="O404" t="inlineStr">
         <is>
@@ -30875,15 +30795,11 @@
           <t>平安航旅</t>
         </is>
       </c>
-      <c r="C405" t="inlineStr">
-        <is>
-          <t>4470</t>
-        </is>
-      </c>
-      <c r="D405" t="inlineStr">
-        <is>
-          <t>138001</t>
-        </is>
+      <c r="C405" t="n">
+        <v>4470</v>
+      </c>
+      <c r="D405" t="n">
+        <v>138001</v>
       </c>
       <c r="E405" t="inlineStr">
         <is>
@@ -30905,35 +30821,23 @@
           <t>系统异常,业务异常,未知异常</t>
         </is>
       </c>
-      <c r="I405" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="J405" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="K405" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="L405" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="M405" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="N405" t="inlineStr">
-        <is>
-          <t>45</t>
-        </is>
+      <c r="I405" t="n">
+        <v>60</v>
+      </c>
+      <c r="J405" t="n">
+        <v>25</v>
+      </c>
+      <c r="K405" t="n">
+        <v>7</v>
+      </c>
+      <c r="L405" t="n">
+        <v>28</v>
+      </c>
+      <c r="M405" t="n">
+        <v>20</v>
+      </c>
+      <c r="N405" t="n">
+        <v>45</v>
       </c>
       <c r="O405" t="inlineStr">
         <is>
@@ -30967,15 +30871,11 @@
           <t>平安航旅</t>
         </is>
       </c>
-      <c r="C406" t="inlineStr">
-        <is>
-          <t>4470</t>
-        </is>
-      </c>
-      <c r="D406" t="inlineStr">
-        <is>
-          <t>138001</t>
-        </is>
+      <c r="C406" t="n">
+        <v>4470</v>
+      </c>
+      <c r="D406" t="n">
+        <v>138001</v>
       </c>
       <c r="E406" t="inlineStr">
         <is>
@@ -30997,35 +30897,23 @@
           <t>系统异常,业务异常,未知异常</t>
         </is>
       </c>
-      <c r="I406" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="J406" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
-      <c r="K406" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="L406" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="M406" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="N406" t="inlineStr">
-        <is>
-          <t>45</t>
-        </is>
+      <c r="I406" t="n">
+        <v>60</v>
+      </c>
+      <c r="J406" t="n">
+        <v>29</v>
+      </c>
+      <c r="K406" t="n">
+        <v>5</v>
+      </c>
+      <c r="L406" t="n">
+        <v>17</v>
+      </c>
+      <c r="M406" t="n">
+        <v>15</v>
+      </c>
+      <c r="N406" t="n">
+        <v>45</v>
       </c>
       <c r="O406" t="inlineStr">
         <is>
@@ -31059,15 +30947,11 @@
           <t>向上航服</t>
         </is>
       </c>
-      <c r="C407" t="inlineStr">
-        <is>
-          <t>5184</t>
-        </is>
-      </c>
-      <c r="D407" t="inlineStr">
-        <is>
-          <t>100745</t>
-        </is>
+      <c r="C407" t="n">
+        <v>5184</v>
+      </c>
+      <c r="D407" t="n">
+        <v>100745</v>
       </c>
       <c r="E407" t="inlineStr">
         <is>
@@ -31089,35 +30973,23 @@
           <t>系统异常,业务异常,未知异常</t>
         </is>
       </c>
-      <c r="I407" t="inlineStr">
-        <is>
-          <t>120</t>
-        </is>
-      </c>
-      <c r="J407" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="K407" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="L407" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="M407" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="N407" t="inlineStr">
-        <is>
-          <t>45</t>
-        </is>
+      <c r="I407" t="n">
+        <v>120</v>
+      </c>
+      <c r="J407" t="n">
+        <v>23</v>
+      </c>
+      <c r="K407" t="n">
+        <v>4</v>
+      </c>
+      <c r="L407" t="n">
+        <v>17</v>
+      </c>
+      <c r="M407" t="n">
+        <v>15</v>
+      </c>
+      <c r="N407" t="n">
+        <v>45</v>
       </c>
       <c r="O407" t="inlineStr">
         <is>
@@ -31151,84 +31023,528 @@
           <t>平安航旅</t>
         </is>
       </c>
-      <c r="C408" t="inlineStr">
+      <c r="C408" t="n">
+        <v>4470</v>
+      </c>
+      <c r="D408" t="n">
+        <v>138001</v>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>QW,DZ,8L,CA,JD,EU,MF,GS,HO,KY,GS,AQ,PN,JD,GJ,HU,9C,Y8,FU</t>
+        </is>
+      </c>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t>9C</t>
+        </is>
+      </c>
+      <c r="G408" t="inlineStr">
+        <is>
+          <t>验座</t>
+        </is>
+      </c>
+      <c r="H408" t="inlineStr">
+        <is>
+          <t>系统异常,业务异常,未知异常</t>
+        </is>
+      </c>
+      <c r="I408" t="n">
+        <v>60</v>
+      </c>
+      <c r="J408" t="n">
+        <v>40</v>
+      </c>
+      <c r="K408" t="n">
+        <v>9</v>
+      </c>
+      <c r="L408" t="n">
+        <v>22</v>
+      </c>
+      <c r="M408" t="n">
+        <v>20</v>
+      </c>
+      <c r="N408" t="n">
+        <v>45</v>
+      </c>
+      <c r="O408" t="inlineStr">
+        <is>
+          <t>2026-10-20 15:37:20</t>
+        </is>
+      </c>
+      <c r="P408" t="inlineStr">
+        <is>
+          <t>2026-10-20 16:22:20</t>
+        </is>
+      </c>
+      <c r="Q408" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:05:57</t>
+        </is>
+      </c>
+      <c r="R408" t="inlineStr">
+        <is>
+          <t>规则id：2 店铺：平安航旅 agentId：4470 channelId：138001 店铺支持销售航司：QW,DZ,8L,CA,JD,EU,MF,GS,HO,KY,GS,AQ,PN,JD,GJ,HU,9C,Y8,FU 下线航司：9C 接口：验座 错误类型：系统异常,业务异常,未知异常 近[ 60 ]分钟内，请求[ 40 ]个，错误[9 ]个。失败率[ 22% ]，高于要求[ 20% ] 下线[45]分钟，屏蔽时间从2026-10-20 15:37:20到2026-10-20 16:22:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>平安航旅</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
         <is>
           <t>4470</t>
         </is>
       </c>
-      <c r="D408" t="inlineStr">
+      <c r="D409" t="inlineStr">
         <is>
           <t>138001</t>
         </is>
       </c>
-      <c r="E408" t="inlineStr">
+      <c r="E409" t="inlineStr">
         <is>
           <t>QW,DZ,8L,CA,JD,EU,MF,GS,HO,KY,GS,AQ,PN,JD,GJ,HU,9C,Y8,FU</t>
         </is>
       </c>
-      <c r="F408" t="inlineStr">
+      <c r="F409" t="inlineStr">
         <is>
           <t>9C</t>
         </is>
       </c>
-      <c r="G408" t="inlineStr">
+      <c r="G409" t="inlineStr">
         <is>
           <t>验座</t>
         </is>
       </c>
-      <c r="H408" t="inlineStr">
-        <is>
-          <t>系统异常,业务异常,未知异常</t>
-        </is>
-      </c>
-      <c r="I408" t="inlineStr">
+      <c r="H409" t="inlineStr">
+        <is>
+          <t>系统异常,业务异常,未知异常</t>
+        </is>
+      </c>
+      <c r="I409" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="J409" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="K409" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="L409" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="M409" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="N409" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="O409" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:41:45</t>
+        </is>
+      </c>
+      <c r="P409" t="inlineStr">
+        <is>
+          <t>2026-10-20 21:11:45</t>
+        </is>
+      </c>
+      <c r="Q409" t="inlineStr">
+        <is>
+          <t>2026-10-21 08:01:01</t>
+        </is>
+      </c>
+      <c r="R409" t="inlineStr">
+        <is>
+          <t>规则id：10 店铺：平安航旅 agentId：4470 channelId：138001 店铺支持销售航司：QW,DZ,8L,CA,JD,EU,MF,GS,HO,KY,GS,AQ,PN,JD,GJ,HU,9C,Y8,FU 下线航司：9C 接口：验座 错误类型：系统异常,业务异常,未知异常 近[ 120 ]分钟内，请求[ 21 ]个，错误[6 ]个。失败率[ 28% ]，高于要求[ 20% ] 由于连续满足下线规则，下线时间延长。下线[90]分钟，屏蔽时间从2026-10-20 19:41:45到2026-10-20 21:11:45 点此查看接口质量明细  自定义 2026年10月20日 21:46 [新版国内大卖家下线通知]</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>平安航旅</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>4470</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>138001</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>QW,DZ,8L,CA,JD,EU,MF,GS,HO,KY,GS,AQ,PN,JD,GJ,HU,9C,Y8,FU</t>
+        </is>
+      </c>
+      <c r="F410" t="inlineStr">
+        <is>
+          <t>9C</t>
+        </is>
+      </c>
+      <c r="G410" t="inlineStr">
+        <is>
+          <t>验座</t>
+        </is>
+      </c>
+      <c r="H410" t="inlineStr">
+        <is>
+          <t>系统异常,业务异常,未知异常</t>
+        </is>
+      </c>
+      <c r="I410" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="J410" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="K410" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="L410" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="M410" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="N410" t="inlineStr">
+        <is>
+          <t>180</t>
+        </is>
+      </c>
+      <c r="O410" t="inlineStr">
+        <is>
+          <t>2026-10-20 21:46:13</t>
+        </is>
+      </c>
+      <c r="P410" t="inlineStr">
+        <is>
+          <t>2026-10-21 00:46:13</t>
+        </is>
+      </c>
+      <c r="Q410" t="inlineStr">
+        <is>
+          <t>2026-10-21 08:01:01</t>
+        </is>
+      </c>
+      <c r="R410" t="inlineStr">
+        <is>
+          <t>规则id：10 店铺：平安航旅 agentId：4470 channelId：138001 店铺支持销售航司：QW,DZ,8L,CA,JD,EU,MF,GS,HO,KY,GS,AQ,PN,JD,GJ,HU,9C,Y8,FU 下线航司：9C 接口：验座 错误类型：系统异常,业务异常,未知异常 近[ 120 ]分钟内，请求[ 21 ]个，错误[7 ]个。失败率[ 33% ]，高于要求[ 20% ] 由于连续满足下线规则，下线时间延长。下线[180]分钟，屏蔽时间从2026-10-20 21:46:13到2026-10-21 00:46:13 点此查看接口质量明细  自定义 2026年10月20日 22:08 [新版国内大卖家下线通知]</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>平安航旅</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>4470</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>138001</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>QW,DZ,8L,CA,JD,EU,MF,GS,HO,KY,GS,AQ,PN,JD,GJ,HU,9C,Y8,FU</t>
+        </is>
+      </c>
+      <c r="F411" t="inlineStr">
+        <is>
+          <t>8L</t>
+        </is>
+      </c>
+      <c r="G411" t="inlineStr">
+        <is>
+          <t>验价</t>
+        </is>
+      </c>
+      <c r="H411" t="inlineStr">
+        <is>
+          <t>系统异常,业务异常,未知异常</t>
+        </is>
+      </c>
+      <c r="I411" t="inlineStr">
         <is>
           <t>60</t>
         </is>
       </c>
-      <c r="J408" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
-      <c r="K408" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="L408" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="M408" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="N408" t="inlineStr">
+      <c r="J411" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="K411" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="L411" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="M411" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="N411" t="inlineStr">
         <is>
           <t>45</t>
         </is>
       </c>
-      <c r="O408" t="inlineStr">
-        <is>
-          <t>2026-10-20 15:37:20</t>
-        </is>
-      </c>
-      <c r="P408" t="inlineStr">
-        <is>
-          <t>2026-10-20 16:22:20</t>
-        </is>
-      </c>
-      <c r="Q408" t="inlineStr">
-        <is>
-          <t>2026-10-20 19:05:57</t>
-        </is>
-      </c>
-      <c r="R408" t="inlineStr">
-        <is>
-          <t>规则id：2 店铺：平安航旅 agentId：4470 channelId：138001 店铺支持销售航司：QW,DZ,8L,CA,JD,EU,MF,GS,HO,KY,GS,AQ,PN,JD,GJ,HU,9C,Y8,FU 下线航司：9C 接口：验座 错误类型：系统异常,业务异常,未知异常 近[ 60 ]分钟内，请求[ 40 ]个，错误[9 ]个。失败率[ 22% ]，高于要求[ 20% ] 下线[45]分钟，屏蔽时间从2026-10-20 15:37:20到2026-10-20 16:22:20</t>
+      <c r="O411" t="inlineStr">
+        <is>
+          <t>2026-10-20 22:08:27</t>
+        </is>
+      </c>
+      <c r="P411" t="inlineStr">
+        <is>
+          <t>2026-10-20 22:53:27</t>
+        </is>
+      </c>
+      <c r="Q411" t="inlineStr">
+        <is>
+          <t>2026-10-21 08:01:01</t>
+        </is>
+      </c>
+      <c r="R411" t="inlineStr">
+        <is>
+          <t>规则id：4 店铺：平安航旅 agentId：4470 channelId：138001 店铺支持销售航司：QW,DZ,8L,CA,JD,EU,MF,GS,HO,KY,GS,AQ,PN,JD,GJ,HU,9C,Y8,FU 下线航司：8L 接口：验价 错误类型：系统异常,业务异常,未知异常 近[ 60 ]分钟内，请求[ 79 ]个，错误[13 ]个。失败率[ 16% ]，高于要求[ 15% ] 下线[45]分钟，屏蔽时间从2026-10-20 22:08:27到2026-10-20 22:53:27 点此查看接口质量明细  自定义 2026年10月20日 23:32 [新版国内大卖家下线通知]</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>向上航服</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>5184</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>100745</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>8L,SC,UQ,CZ,AQ,GS,PN,QW,9C,HO,GJ,MF,HU</t>
+        </is>
+      </c>
+      <c r="F412" t="inlineStr">
+        <is>
+          <t>UQ</t>
+        </is>
+      </c>
+      <c r="G412" t="inlineStr">
+        <is>
+          <t>预定</t>
+        </is>
+      </c>
+      <c r="H412" t="inlineStr">
+        <is>
+          <t>系统异常,业务异常,未知异常</t>
+        </is>
+      </c>
+      <c r="I412" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="J412" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="K412" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="L412" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="M412" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="N412" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="O412" t="inlineStr">
+        <is>
+          <t>2026-10-20 23:32:22</t>
+        </is>
+      </c>
+      <c r="P412" t="inlineStr">
+        <is>
+          <t>2026-10-21 00:17:22</t>
+        </is>
+      </c>
+      <c r="Q412" t="inlineStr">
+        <is>
+          <t>2026-10-21 08:01:01</t>
+        </is>
+      </c>
+      <c r="R412" t="inlineStr">
+        <is>
+          <t>规则id：6 店铺：向上航服 agentId：5184 channelId：100745 店铺支持销售航司：8L,SC,UQ,CZ,AQ,GS,PN,QW,9C,HO,GJ,MF,HU 下线航司：UQ 接口：预定 错误类型：系统异常,业务异常,未知异常 近[ 60 ]分钟内，请求[ 31 ]个，错误[5 ]个。失败率[ 16% ]，高于要求[ 15% ] 下线[45]分钟，屏蔽时间从2026-10-20 23:32:22到2026-10-21 00:17:22 点此查看接口质量明细  自定义 2026年10月21日 00:53 [新版国内大卖家下线通知]</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>平安航旅</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>4470</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>138001</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>QW,DZ,8L,CA,JD,EU,MF,GS,HO,KY,GS,AQ,PN,JD,GJ,HU,9C,Y8,FU</t>
+        </is>
+      </c>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="G413" t="inlineStr">
+        <is>
+          <t>预定</t>
+        </is>
+      </c>
+      <c r="H413" t="inlineStr">
+        <is>
+          <t>系统异常,业务异常,未知异常</t>
+        </is>
+      </c>
+      <c r="I413" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="J413" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="K413" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="L413" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="M413" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="N413" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="O413" t="inlineStr">
+        <is>
+          <t>2026-10-21 00:53:57</t>
+        </is>
+      </c>
+      <c r="P413" t="inlineStr">
+        <is>
+          <t>2026-10-21 01:38:57</t>
+        </is>
+      </c>
+      <c r="Q413" t="inlineStr">
+        <is>
+          <t>2026-10-21 08:01:01</t>
+        </is>
+      </c>
+      <c r="R413" t="inlineStr">
+        <is>
+          <t>规则id：14 店铺：平安航旅 agentId：4470 channelId：138001 店铺支持销售航司：QW,DZ,8L,CA,JD,EU,MF,GS,HO,KY,GS,AQ,PN,JD,GJ,HU,9C,Y8,FU 下线航司：KY 接口：预定 错误类型：系统异常,业务异常,未知异常 近[ 120 ]分钟内，请求[ 37 ]个，错误[6 ]个。失败率[ 16% ]，高于要求[ 15% ] 下线[45]分钟，屏蔽时间从2026-10-21 00:53:57到2026-10-21 01:38:57</t>
         </is>
       </c>
     </row>

</xml_diff>